<commit_message>
Mise à jour site
</commit_message>
<xml_diff>
--- a/prix/prix.xlsx
+++ b/prix/prix.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\platres-et-enduits\prix\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3972BC67-59DF-49DB-B649-ACBEA46CA44B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E42F2FB-29ED-4C5A-A59E-F0120410DAC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="23016" yWindow="84" windowWidth="19116" windowHeight="10884" xr2:uid="{6E95DC93-531D-460D-9A06-44397A8920D7}"/>
+    <workbookView xWindow="22656" yWindow="192" windowWidth="19116" windowHeight="10884" xr2:uid="{6E95DC93-531D-460D-9A06-44397A8920D7}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -2150,14 +2150,14 @@
       <c r="C2" s="5" t="s">
         <v>219</v>
       </c>
-      <c r="D2" s="37">
+      <c r="D2" s="35">
         <v>24.26</v>
       </c>
       <c r="E2" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="F2" s="38">
-        <v>6</v>
+      <c r="F2" s="36">
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
@@ -2170,13 +2170,13 @@
       <c r="C3" s="5" t="s">
         <v>220</v>
       </c>
-      <c r="D3" s="37">
+      <c r="D3" s="35">
         <v>23.1</v>
       </c>
       <c r="E3" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="F3" s="38">
+      <c r="F3" s="36">
         <v>5</v>
       </c>
     </row>
@@ -2188,14 +2188,14 @@
       <c r="C4" s="5" t="s">
         <v>221</v>
       </c>
-      <c r="D4" s="37">
+      <c r="D4" s="35">
         <v>7.8</v>
       </c>
       <c r="E4" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="F4" s="38">
-        <v>1</v>
+      <c r="F4" s="36">
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
@@ -2206,14 +2206,14 @@
       <c r="C5" s="5" t="s">
         <v>222</v>
       </c>
-      <c r="D5" s="37">
+      <c r="D5" s="35">
         <v>7.66</v>
       </c>
       <c r="E5" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="F5" s="38">
-        <v>15</v>
+      <c r="F5" s="36">
+        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
@@ -2226,14 +2226,14 @@
       <c r="C6" s="5" t="s">
         <v>226</v>
       </c>
-      <c r="D6" s="37">
+      <c r="D6" s="35">
         <v>17.16</v>
       </c>
       <c r="E6" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="F6" s="38">
-        <v>4</v>
+      <c r="F6" s="36">
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
@@ -2246,14 +2246,14 @@
       <c r="C7" s="5" t="s">
         <v>227</v>
       </c>
-      <c r="D7" s="37">
-        <v>16.830000000000002</v>
+      <c r="D7" s="35">
+        <v>17.64</v>
       </c>
       <c r="E7" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="F7" s="38">
-        <v>2</v>
+      <c r="F7" s="36">
+        <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
@@ -2266,14 +2266,14 @@
       <c r="C8" s="5" t="s">
         <v>223</v>
       </c>
-      <c r="D8" s="37">
-        <v>8.6</v>
+      <c r="D8" s="35">
+        <v>9.0299999999999994</v>
       </c>
       <c r="E8" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="F8" s="38">
-        <v>18</v>
+      <c r="F8" s="36">
+        <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
@@ -2286,14 +2286,14 @@
       <c r="C9" s="5" t="s">
         <v>228</v>
       </c>
-      <c r="D9" s="37">
+      <c r="D9" s="35">
         <v>32.130000000000003</v>
       </c>
       <c r="E9" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="F9" s="38">
-        <v>46</v>
+      <c r="F9" s="36">
+        <v>55</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
@@ -2306,13 +2306,13 @@
       <c r="C10" s="5" t="s">
         <v>229</v>
       </c>
-      <c r="D10" s="37">
+      <c r="D10" s="35">
         <v>33.090000000000003</v>
       </c>
       <c r="E10" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="F10" s="38">
+      <c r="F10" s="36">
         <v>9</v>
       </c>
     </row>
@@ -2324,14 +2324,14 @@
       <c r="C11" s="5" t="s">
         <v>223</v>
       </c>
-      <c r="D11" s="37">
+      <c r="D11" s="35">
         <v>8.86</v>
       </c>
       <c r="E11" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="F11" s="38">
-        <v>-1</v>
+      <c r="F11" s="36">
+        <v>-4</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
@@ -2344,13 +2344,13 @@
       <c r="C12" s="5" t="s">
         <v>230</v>
       </c>
-      <c r="D12" s="37">
+      <c r="D12" s="35">
         <v>19.41</v>
       </c>
       <c r="E12" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="F12" s="38">
+      <c r="F12" s="36">
         <v>1</v>
       </c>
     </row>
@@ -2364,13 +2364,13 @@
       <c r="C13" s="5" t="s">
         <v>231</v>
       </c>
-      <c r="D13" s="37">
+      <c r="D13" s="35">
         <v>65.33</v>
       </c>
       <c r="E13" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="F13" s="38">
+      <c r="F13" s="36">
         <v>3</v>
       </c>
     </row>
@@ -2382,14 +2382,14 @@
       <c r="C14" s="5" t="s">
         <v>223</v>
       </c>
-      <c r="D14" s="37">
+      <c r="D14" s="35">
         <v>11.82</v>
       </c>
       <c r="E14" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="F14" s="38">
-        <v>8</v>
+      <c r="F14" s="36">
+        <v>6</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
@@ -2402,14 +2402,14 @@
       <c r="C15" s="5" t="s">
         <v>223</v>
       </c>
-      <c r="D15" s="37">
+      <c r="D15" s="35">
         <v>35.56</v>
       </c>
       <c r="E15" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="F15" s="38">
-        <v>3</v>
+      <c r="F15" s="36">
+        <v>2</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
@@ -2422,13 +2422,13 @@
       <c r="C16" s="5" t="s">
         <v>229</v>
       </c>
-      <c r="D16" s="37">
+      <c r="D16" s="35">
         <v>89.14</v>
       </c>
       <c r="E16" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="F16" s="38">
+      <c r="F16" s="36">
         <v>4</v>
       </c>
     </row>
@@ -2442,13 +2442,13 @@
       <c r="C17" s="5" t="s">
         <v>230</v>
       </c>
-      <c r="D17" s="37">
+      <c r="D17" s="35">
         <v>24.32</v>
       </c>
       <c r="E17" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="F17" s="38">
+      <c r="F17" s="36">
         <v>4</v>
       </c>
     </row>
@@ -2462,13 +2462,13 @@
       <c r="C18" s="5" t="s">
         <v>224</v>
       </c>
-      <c r="D18" s="37">
+      <c r="D18" s="35">
         <v>31.240000000000002</v>
       </c>
       <c r="E18" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="F18" s="38">
+      <c r="F18" s="36">
         <v>4</v>
       </c>
     </row>
@@ -2482,13 +2482,13 @@
       <c r="C19" s="5" t="s">
         <v>223</v>
       </c>
-      <c r="D19" s="37">
+      <c r="D19" s="35">
         <v>28.82</v>
       </c>
       <c r="E19" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="F19" s="38">
+      <c r="F19" s="36">
         <v>4</v>
       </c>
     </row>
@@ -2502,13 +2502,13 @@
       <c r="C20" s="5" t="s">
         <v>229</v>
       </c>
-      <c r="D20" s="37">
+      <c r="D20" s="35">
         <v>72.710000000000008</v>
       </c>
       <c r="E20" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="F20" s="38">
+      <c r="F20" s="36">
         <v>3</v>
       </c>
     </row>
@@ -2522,13 +2522,13 @@
       <c r="C21" s="5" t="s">
         <v>225</v>
       </c>
-      <c r="D21" s="37">
+      <c r="D21" s="35">
         <v>9.84</v>
       </c>
       <c r="E21" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="F21" s="38">
+      <c r="F21" s="36">
         <v>12</v>
       </c>
     </row>
@@ -2540,13 +2540,13 @@
       <c r="C22" s="5" t="s">
         <v>230</v>
       </c>
-      <c r="D22" s="37">
+      <c r="D22" s="35">
         <v>23.8</v>
       </c>
       <c r="E22" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="F22" s="38">
+      <c r="F22" s="36">
         <v>2</v>
       </c>
     </row>
@@ -2558,13 +2558,13 @@
       <c r="C23" s="5" t="s">
         <v>232</v>
       </c>
-      <c r="D23" s="37">
+      <c r="D23" s="35">
         <v>35.68</v>
       </c>
       <c r="E23" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="F23" s="38">
+      <c r="F23" s="36">
         <v>0</v>
       </c>
     </row>
@@ -2576,14 +2576,14 @@
       <c r="C24" s="5" t="s">
         <v>233</v>
       </c>
-      <c r="D24" s="37">
-        <v>18.22</v>
+      <c r="D24" s="35">
+        <v>19.48</v>
       </c>
       <c r="E24" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="F24" s="38">
-        <v>6</v>
+      <c r="F24" s="36">
+        <v>10</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
@@ -2594,13 +2594,13 @@
       <c r="C25" s="5" t="s">
         <v>234</v>
       </c>
-      <c r="D25" s="37">
+      <c r="D25" s="35">
         <v>18.150000000000002</v>
       </c>
       <c r="E25" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="F25" s="38">
+      <c r="F25" s="36">
         <v>1</v>
       </c>
     </row>
@@ -2614,13 +2614,13 @@
       <c r="C26" s="5" t="s">
         <v>236</v>
       </c>
-      <c r="D26" s="37">
+      <c r="D26" s="35">
         <v>15.63</v>
       </c>
       <c r="E26" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="F26" s="38">
+      <c r="F26" s="36">
         <v>15</v>
       </c>
     </row>
@@ -2634,13 +2634,13 @@
       <c r="C27" s="5" t="s">
         <v>228</v>
       </c>
-      <c r="D27" s="37">
+      <c r="D27" s="35">
         <v>29.5</v>
       </c>
       <c r="E27" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="F27" s="38">
+      <c r="F27" s="36">
         <v>3</v>
       </c>
     </row>
@@ -2654,14 +2654,14 @@
       <c r="C28" s="5" t="s">
         <v>228</v>
       </c>
-      <c r="D28" s="37">
+      <c r="D28" s="35">
         <v>49.51</v>
       </c>
       <c r="E28" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="F28" s="38">
-        <v>17</v>
+      <c r="F28" s="36">
+        <v>22</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
@@ -2674,13 +2674,13 @@
       <c r="C29" s="5" t="s">
         <v>235</v>
       </c>
-      <c r="D29" s="37">
+      <c r="D29" s="35">
         <v>64</v>
       </c>
       <c r="E29" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="F29" s="38">
+      <c r="F29" s="36">
         <v>1</v>
       </c>
     </row>
@@ -2692,13 +2692,13 @@
       <c r="C30" s="5" t="s">
         <v>223</v>
       </c>
-      <c r="D30" s="37">
+      <c r="D30" s="35">
         <v>18.37</v>
       </c>
       <c r="E30" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="F30" s="38">
+      <c r="F30" s="36">
         <v>0</v>
       </c>
     </row>
@@ -2710,13 +2710,13 @@
       <c r="C31" s="5" t="s">
         <v>229</v>
       </c>
-      <c r="D31" s="37">
+      <c r="D31" s="35">
         <v>39.57</v>
       </c>
       <c r="E31" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="F31" s="38">
+      <c r="F31" s="36">
         <v>-1</v>
       </c>
     </row>
@@ -2730,13 +2730,13 @@
       <c r="C32" s="5" t="s">
         <v>228</v>
       </c>
-      <c r="D32" s="37">
+      <c r="D32" s="35">
         <v>44.78</v>
       </c>
       <c r="E32" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="F32" s="38">
+      <c r="F32" s="36">
         <v>0</v>
       </c>
     </row>
@@ -2748,13 +2748,13 @@
       <c r="C33" s="5" t="s">
         <v>228</v>
       </c>
-      <c r="D33" s="37">
+      <c r="D33" s="35">
         <v>44.61</v>
       </c>
       <c r="E33" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="F33" s="38">
+      <c r="F33" s="36">
         <v>3</v>
       </c>
     </row>
@@ -2766,13 +2766,13 @@
       <c r="C34" s="5" t="s">
         <v>231</v>
       </c>
-      <c r="D34" s="37">
+      <c r="D34" s="35">
         <v>25.22</v>
       </c>
       <c r="E34" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="F34" s="38">
+      <c r="F34" s="36">
         <v>1</v>
       </c>
     </row>
@@ -2784,13 +2784,13 @@
       <c r="C35" s="5" t="s">
         <v>237</v>
       </c>
-      <c r="D35" s="37">
+      <c r="D35" s="35">
         <v>52.01</v>
       </c>
       <c r="E35" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="F35" s="38">
+      <c r="F35" s="36">
         <v>2</v>
       </c>
     </row>
@@ -2802,13 +2802,13 @@
       <c r="C36" s="5" t="s">
         <v>224</v>
       </c>
-      <c r="D36" s="37">
+      <c r="D36" s="35">
         <v>24.32</v>
       </c>
       <c r="E36" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="F36" s="38">
+      <c r="F36" s="36">
         <v>5</v>
       </c>
     </row>
@@ -2822,14 +2822,14 @@
       <c r="C37" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="D37" s="39">
+      <c r="D37" s="37">
         <v>15.06</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="F37" s="40">
-        <v>35</v>
+      <c r="F37" s="38">
+        <v>10</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
@@ -2842,14 +2842,14 @@
       <c r="C38" s="5" t="s">
         <v>238</v>
       </c>
-      <c r="D38" s="39">
+      <c r="D38" s="37">
         <v>9.57</v>
       </c>
       <c r="E38" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="F38" s="40">
-        <v>20</v>
+      <c r="F38" s="38">
+        <v>14</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
@@ -2862,14 +2862,14 @@
       <c r="C39" s="5" t="s">
         <v>228</v>
       </c>
-      <c r="D39" s="39">
+      <c r="D39" s="37">
         <v>13.65</v>
       </c>
       <c r="E39" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="F39" s="40">
-        <v>57</v>
+      <c r="F39" s="38">
+        <v>51</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
@@ -2882,14 +2882,14 @@
       <c r="C40" s="5" t="s">
         <v>228</v>
       </c>
-      <c r="D40" s="39">
-        <v>12.86</v>
+      <c r="D40" s="37">
+        <v>12.9</v>
       </c>
       <c r="E40" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="F40" s="40">
-        <v>448</v>
+      <c r="F40" s="38">
+        <v>399</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
@@ -2902,14 +2902,14 @@
       <c r="C41" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="D41" s="39">
-        <v>18.21</v>
+      <c r="D41" s="37">
+        <v>19.59</v>
       </c>
       <c r="E41" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="F41" s="40">
-        <v>20</v>
+      <c r="F41" s="38">
+        <v>33</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
@@ -2922,14 +2922,14 @@
       <c r="C42" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="D42" s="39">
+      <c r="D42" s="37">
         <v>16.48</v>
       </c>
       <c r="E42" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="F42" s="40">
-        <v>60</v>
+      <c r="F42" s="38">
+        <v>29</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
@@ -2949,7 +2949,7 @@
         <v>12</v>
       </c>
       <c r="F43" s="5">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
@@ -2969,7 +2969,7 @@
         <v>13</v>
       </c>
       <c r="F44" s="5">
-        <v>87</v>
+        <v>60</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
@@ -2983,13 +2983,13 @@
         <v>228</v>
       </c>
       <c r="D45" s="3">
-        <v>21.89</v>
+        <v>21.93</v>
       </c>
       <c r="E45" s="16" t="s">
         <v>14</v>
       </c>
       <c r="F45" s="5">
-        <v>26</v>
+        <v>56</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
@@ -3009,7 +3009,7 @@
         <v>15</v>
       </c>
       <c r="F46" s="5">
-        <v>13</v>
+        <v>6</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
@@ -3022,14 +3022,14 @@
       <c r="C47" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="D47" s="41">
+      <c r="D47" s="39">
         <v>5.5200000000000005</v>
       </c>
       <c r="E47" s="17" t="s">
         <v>103</v>
       </c>
-      <c r="F47" s="42">
-        <v>230.40000000000003</v>
+      <c r="F47" s="40">
+        <v>229.60000000000002</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
@@ -3042,14 +3042,14 @@
       <c r="C48" s="2" t="s">
         <v>241</v>
       </c>
-      <c r="D48" s="41">
+      <c r="D48" s="39">
         <v>5.25</v>
       </c>
       <c r="E48" s="17" t="s">
         <v>104</v>
       </c>
-      <c r="F48" s="42">
-        <v>321.36</v>
+      <c r="F48" s="40">
+        <v>312</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
@@ -3062,14 +3062,14 @@
       <c r="C49" s="2" t="s">
         <v>242</v>
       </c>
-      <c r="D49" s="41">
-        <v>4.74</v>
+      <c r="D49" s="39">
+        <v>5.25</v>
       </c>
       <c r="E49" s="17" t="s">
         <v>105</v>
       </c>
-      <c r="F49" s="42">
-        <v>265.32000000000028</v>
+      <c r="F49" s="40">
+        <v>276.24000000000029</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
@@ -3082,14 +3082,14 @@
       <c r="C50" s="2" t="s">
         <v>247</v>
       </c>
-      <c r="D50" s="41">
-        <v>4.66</v>
+      <c r="D50" s="39">
+        <v>5.07</v>
       </c>
       <c r="E50" s="17" t="s">
         <v>106</v>
       </c>
-      <c r="F50" s="42">
-        <v>377.17999999999972</v>
+      <c r="F50" s="40">
+        <v>179.12999999999977</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
@@ -3102,13 +3102,13 @@
       <c r="C51" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="D51" s="41">
+      <c r="D51" s="39">
         <v>5.26</v>
       </c>
       <c r="E51" s="17" t="s">
         <v>107</v>
       </c>
-      <c r="F51" s="42">
+      <c r="F51" s="40">
         <v>0</v>
       </c>
     </row>
@@ -3122,14 +3122,14 @@
       <c r="C52" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="D52" s="41">
+      <c r="D52" s="39">
         <v>2.65</v>
       </c>
       <c r="E52" s="17" t="s">
         <v>108</v>
       </c>
-      <c r="F52" s="42">
-        <v>472.67999999999915</v>
+      <c r="F52" s="40">
+        <v>403.51999999999913</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.3">
@@ -3142,13 +3142,13 @@
       <c r="C53" s="2" t="s">
         <v>245</v>
       </c>
-      <c r="D53" s="41">
+      <c r="D53" s="39">
         <v>5.26</v>
       </c>
       <c r="E53" s="17" t="s">
         <v>109</v>
       </c>
-      <c r="F53" s="42">
+      <c r="F53" s="40">
         <v>6.7199999999999758</v>
       </c>
     </row>
@@ -3162,13 +3162,13 @@
       <c r="C54" s="2" t="s">
         <v>246</v>
       </c>
-      <c r="D54" s="41">
+      <c r="D54" s="39">
         <v>5.13</v>
       </c>
       <c r="E54" s="17" t="s">
         <v>110</v>
       </c>
-      <c r="F54" s="42">
+      <c r="F54" s="40">
         <v>0</v>
       </c>
     </row>
@@ -3182,14 +3182,14 @@
       <c r="C55" s="2" t="s">
         <v>248</v>
       </c>
-      <c r="D55" s="41">
+      <c r="D55" s="39">
         <v>4.83</v>
       </c>
       <c r="E55" s="17" t="s">
         <v>111</v>
       </c>
-      <c r="F55" s="42">
-        <v>298.14199999999801</v>
+      <c r="F55" s="40">
+        <v>13.421999999997894</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.3">
@@ -3202,14 +3202,14 @@
       <c r="C56" s="2" t="s">
         <v>248</v>
       </c>
-      <c r="D56" s="41">
+      <c r="D56" s="39">
         <v>8.18</v>
       </c>
       <c r="E56" s="17" t="s">
         <v>112</v>
       </c>
-      <c r="F56" s="42">
-        <v>254.29999999999907</v>
+      <c r="F56" s="40">
+        <v>163.89999999999901</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.3">
@@ -3222,14 +3222,14 @@
       <c r="C57" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="D57" s="41">
+      <c r="D57" s="39">
         <v>8.48</v>
       </c>
       <c r="E57" s="17" t="s">
         <v>113</v>
       </c>
-      <c r="F57" s="42">
-        <v>298.52000000000089</v>
+      <c r="F57" s="40">
+        <v>225.72000000000088</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.3">
@@ -3242,13 +3242,13 @@
       <c r="C58" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="D58" s="41">
+      <c r="D58" s="39">
         <v>7.25</v>
       </c>
       <c r="E58" s="17" t="s">
         <v>114</v>
       </c>
-      <c r="F58" s="42">
+      <c r="F58" s="40">
         <v>0</v>
       </c>
     </row>
@@ -3262,13 +3262,13 @@
       <c r="C59" s="2" t="s">
         <v>249</v>
       </c>
-      <c r="D59" s="41">
+      <c r="D59" s="39">
         <v>8.1300000000000008</v>
       </c>
       <c r="E59" s="17" t="s">
         <v>115</v>
       </c>
-      <c r="F59" s="42">
+      <c r="F59" s="40">
         <v>115.43999999999997</v>
       </c>
     </row>
@@ -3282,14 +3282,14 @@
       <c r="C60" s="2" t="s">
         <v>250</v>
       </c>
-      <c r="D60" s="41">
+      <c r="D60" s="39">
         <v>8.43</v>
       </c>
       <c r="E60" s="17" t="s">
         <v>116</v>
       </c>
-      <c r="F60" s="42">
-        <v>85.799999999999969</v>
+      <c r="F60" s="40">
+        <v>3.1199999999999641</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.3">
@@ -3302,14 +3302,14 @@
       <c r="C61" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="D61" s="41">
+      <c r="D61" s="39">
         <v>8.4499999999999993</v>
       </c>
       <c r="E61" s="17" t="s">
         <v>117</v>
       </c>
-      <c r="F61" s="42">
-        <v>84.240000000000109</v>
+      <c r="F61" s="40">
+        <v>15.600000000000101</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.3">
@@ -3322,13 +3322,13 @@
       <c r="C62" s="2" t="s">
         <v>248</v>
       </c>
-      <c r="D62" s="41">
+      <c r="D62" s="39">
         <v>9.33</v>
       </c>
       <c r="E62" s="17" t="s">
         <v>118</v>
       </c>
-      <c r="F62" s="42">
+      <c r="F62" s="40">
         <v>0</v>
       </c>
     </row>
@@ -3342,14 +3342,14 @@
       <c r="C63" s="2" t="s">
         <v>251</v>
       </c>
-      <c r="D63" s="43">
-        <v>23.900000000000002</v>
+      <c r="D63" s="41">
+        <v>25.6</v>
       </c>
       <c r="E63" s="21" t="s">
         <v>135</v>
       </c>
-      <c r="F63" s="44">
-        <v>7</v>
+      <c r="F63" s="42">
+        <v>26</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.3">
@@ -3362,14 +3362,14 @@
       <c r="C64" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="D64" s="43">
-        <v>11.120000000000001</v>
+      <c r="D64" s="41">
+        <v>11.66</v>
       </c>
       <c r="E64" s="21" t="s">
         <v>136</v>
       </c>
-      <c r="F64" s="44">
-        <v>4</v>
+      <c r="F64" s="42">
+        <v>10</v>
       </c>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.3">
@@ -3382,14 +3382,14 @@
       <c r="C65" s="2" t="s">
         <v>253</v>
       </c>
-      <c r="D65" s="43">
+      <c r="D65" s="41">
         <v>12.58</v>
       </c>
       <c r="E65" s="21" t="s">
         <v>137</v>
       </c>
-      <c r="F65" s="44">
-        <v>12</v>
+      <c r="F65" s="42">
+        <v>9</v>
       </c>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.3">
@@ -3402,14 +3402,14 @@
       <c r="C66" s="2" t="s">
         <v>254</v>
       </c>
-      <c r="D66" s="43">
+      <c r="D66" s="41">
         <v>1.84</v>
       </c>
       <c r="E66" s="21" t="s">
         <v>138</v>
       </c>
-      <c r="F66" s="44">
-        <v>22</v>
+      <c r="F66" s="42">
+        <v>6</v>
       </c>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.3">
@@ -3422,14 +3422,14 @@
       <c r="C67" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="D67" s="43">
+      <c r="D67" s="41">
         <v>5.72</v>
       </c>
       <c r="E67" s="21" t="s">
         <v>139</v>
       </c>
-      <c r="F67" s="44">
-        <v>0</v>
+      <c r="F67" s="42">
+        <v>61</v>
       </c>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.3">
@@ -3440,13 +3440,13 @@
       <c r="C68" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="D68" s="43">
+      <c r="D68" s="41">
         <v>5</v>
       </c>
       <c r="E68" s="21" t="s">
         <v>140</v>
       </c>
-      <c r="F68" s="44">
+      <c r="F68" s="42">
         <v>0</v>
       </c>
     </row>
@@ -3460,13 +3460,13 @@
       <c r="C69" s="2" t="s">
         <v>256</v>
       </c>
-      <c r="D69" s="43">
+      <c r="D69" s="41">
         <v>5.49</v>
       </c>
       <c r="E69" s="21" t="s">
         <v>141</v>
       </c>
-      <c r="F69" s="44">
+      <c r="F69" s="42">
         <v>0</v>
       </c>
     </row>
@@ -3478,13 +3478,13 @@
       <c r="C70" s="2" t="s">
         <v>257</v>
       </c>
-      <c r="D70" s="43">
+      <c r="D70" s="41">
         <v>19.41</v>
       </c>
       <c r="E70" s="21" t="s">
         <v>142</v>
       </c>
-      <c r="F70" s="44">
+      <c r="F70" s="42">
         <v>0</v>
       </c>
     </row>
@@ -3498,14 +3498,14 @@
       <c r="C71" s="2" t="s">
         <v>258</v>
       </c>
-      <c r="D71" s="45">
-        <v>25.8</v>
+      <c r="D71" s="43">
+        <v>22.09</v>
       </c>
       <c r="E71" s="22" t="s">
         <v>151</v>
       </c>
-      <c r="F71" s="46">
-        <v>1</v>
+      <c r="F71" s="44">
+        <v>4</v>
       </c>
       <c r="G71" s="19"/>
     </row>
@@ -3519,13 +3519,13 @@
       <c r="C72" s="2" t="s">
         <v>259</v>
       </c>
-      <c r="D72" s="45">
+      <c r="D72" s="43">
         <v>27.3</v>
       </c>
       <c r="E72" s="22" t="s">
         <v>152</v>
       </c>
-      <c r="F72" s="46">
+      <c r="F72" s="44">
         <v>0</v>
       </c>
     </row>
@@ -3539,14 +3539,14 @@
       <c r="C73" s="2" t="s">
         <v>260</v>
       </c>
-      <c r="D73" s="45">
-        <v>40.119999999999997</v>
+      <c r="D73" s="43">
+        <v>34.869999999999997</v>
       </c>
       <c r="E73" s="22" t="s">
         <v>153</v>
       </c>
-      <c r="F73" s="46">
-        <v>5</v>
+      <c r="F73" s="44">
+        <v>6</v>
       </c>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.3">
@@ -3559,14 +3559,14 @@
       <c r="C74" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="D74" s="45">
+      <c r="D74" s="43">
         <v>16.170000000000002</v>
       </c>
       <c r="E74" s="22" t="s">
         <v>154</v>
       </c>
-      <c r="F74" s="46">
-        <v>7</v>
+      <c r="F74" s="44">
+        <v>3</v>
       </c>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.3">
@@ -3579,14 +3579,14 @@
       <c r="C75" s="2" t="s">
         <v>262</v>
       </c>
-      <c r="D75" s="45">
+      <c r="D75" s="43">
         <v>22.05</v>
       </c>
       <c r="E75" s="22" t="s">
         <v>155</v>
       </c>
-      <c r="F75" s="46">
-        <v>3</v>
+      <c r="F75" s="44">
+        <v>8</v>
       </c>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.3">
@@ -3599,13 +3599,13 @@
       <c r="C76" s="2" t="s">
         <v>263</v>
       </c>
-      <c r="D76" s="45">
+      <c r="D76" s="43">
         <v>25.810000000000002</v>
       </c>
       <c r="E76" s="22" t="s">
         <v>156</v>
       </c>
-      <c r="F76" s="46">
+      <c r="F76" s="44">
         <v>6</v>
       </c>
     </row>
@@ -3619,14 +3619,14 @@
       <c r="C77" s="2" t="s">
         <v>264</v>
       </c>
-      <c r="D77" s="45">
-        <v>13.07</v>
+      <c r="D77" s="43">
+        <v>13.43</v>
       </c>
       <c r="E77" s="22" t="s">
         <v>157</v>
       </c>
-      <c r="F77" s="46">
-        <v>18</v>
+      <c r="F77" s="44">
+        <v>13</v>
       </c>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.3">
@@ -3639,14 +3639,14 @@
       <c r="C78" s="2" t="s">
         <v>265</v>
       </c>
-      <c r="D78" s="45">
+      <c r="D78" s="43">
         <v>3.22</v>
       </c>
       <c r="E78" s="22" t="s">
         <v>158</v>
       </c>
-      <c r="F78" s="46">
-        <v>9</v>
+      <c r="F78" s="44">
+        <v>6</v>
       </c>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.3">
@@ -3659,13 +3659,13 @@
       <c r="C79" s="5" t="s">
         <v>266</v>
       </c>
-      <c r="D79" s="45">
+      <c r="D79" s="43">
         <v>16.63</v>
       </c>
       <c r="E79" s="22" t="s">
         <v>159</v>
       </c>
-      <c r="F79" s="46">
+      <c r="F79" s="44">
         <v>36</v>
       </c>
     </row>
@@ -3679,14 +3679,14 @@
       <c r="C80" s="5" t="s">
         <v>267</v>
       </c>
-      <c r="D80" s="45">
-        <v>6.36</v>
+      <c r="D80" s="43">
+        <v>6.53</v>
       </c>
       <c r="E80" s="22" t="s">
         <v>160</v>
       </c>
-      <c r="F80" s="46">
-        <v>12</v>
+      <c r="F80" s="44">
+        <v>21</v>
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.3">
@@ -3699,14 +3699,14 @@
       <c r="C81" s="5" t="s">
         <v>268</v>
       </c>
-      <c r="D81" s="45">
-        <v>15.73</v>
+      <c r="D81" s="43">
+        <v>24.830000000000002</v>
       </c>
       <c r="E81" s="22" t="s">
         <v>161</v>
       </c>
-      <c r="F81" s="46">
-        <v>-10</v>
+      <c r="F81" s="44">
+        <v>-5</v>
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.3">
@@ -3719,14 +3719,14 @@
       <c r="C82" s="5" t="s">
         <v>266</v>
       </c>
-      <c r="D82" s="45">
-        <v>3.92</v>
+      <c r="D82" s="43">
+        <v>6.53</v>
       </c>
       <c r="E82" s="22" t="s">
         <v>162</v>
       </c>
-      <c r="F82" s="46">
-        <v>10</v>
+      <c r="F82" s="44">
+        <v>9</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.3">
@@ -3739,14 +3739,14 @@
       <c r="C83" s="5" t="s">
         <v>269</v>
       </c>
-      <c r="D83" s="45">
-        <v>21.95</v>
+      <c r="D83" s="43">
+        <v>22.55</v>
       </c>
       <c r="E83" s="22" t="s">
         <v>163</v>
       </c>
-      <c r="F83" s="46">
-        <v>2</v>
+      <c r="F83" s="44">
+        <v>8</v>
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.3">
@@ -3759,14 +3759,14 @@
       <c r="C84" s="5" t="s">
         <v>269</v>
       </c>
-      <c r="D84" s="45">
+      <c r="D84" s="43">
         <v>4.99</v>
       </c>
       <c r="E84" s="22" t="s">
         <v>164</v>
       </c>
-      <c r="F84" s="46">
-        <v>8</v>
+      <c r="F84" s="44">
+        <v>2</v>
       </c>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.3">
@@ -3779,13 +3779,13 @@
       <c r="C85" s="5" t="s">
         <v>269</v>
       </c>
-      <c r="D85" s="45">
-        <v>7.36</v>
+      <c r="D85" s="43">
+        <v>7.7700000000000005</v>
       </c>
       <c r="E85" s="22" t="s">
         <v>165</v>
       </c>
-      <c r="F85" s="46">
+      <c r="F85" s="44">
         <v>19</v>
       </c>
     </row>
@@ -3799,14 +3799,14 @@
       <c r="C86" s="5" t="s">
         <v>270</v>
       </c>
-      <c r="D86" s="45">
+      <c r="D86" s="43">
         <v>30.52</v>
       </c>
       <c r="E86" s="22" t="s">
         <v>166</v>
       </c>
-      <c r="F86" s="46">
-        <v>6</v>
+      <c r="F86" s="44">
+        <v>5</v>
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.3">
@@ -3819,13 +3819,13 @@
       <c r="C87" s="5" t="s">
         <v>271</v>
       </c>
-      <c r="D87" s="45">
+      <c r="D87" s="43">
         <v>6.05</v>
       </c>
       <c r="E87" s="22" t="s">
         <v>167</v>
       </c>
-      <c r="F87" s="46">
+      <c r="F87" s="44">
         <v>11</v>
       </c>
     </row>
@@ -3839,14 +3839,14 @@
       <c r="C88" s="5" t="s">
         <v>271</v>
       </c>
-      <c r="D88" s="45">
+      <c r="D88" s="43">
         <v>4.67</v>
       </c>
       <c r="E88" s="22" t="s">
         <v>168</v>
       </c>
-      <c r="F88" s="46">
-        <v>5</v>
+      <c r="F88" s="44">
+        <v>4</v>
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.3">
@@ -3859,13 +3859,13 @@
       <c r="C89" s="5" t="s">
         <v>259</v>
       </c>
-      <c r="D89" s="45">
+      <c r="D89" s="43">
         <v>15.58</v>
       </c>
       <c r="E89" s="22" t="s">
         <v>169</v>
       </c>
-      <c r="F89" s="46">
+      <c r="F89" s="44">
         <v>0</v>
       </c>
     </row>
@@ -3879,13 +3879,13 @@
       <c r="C90" s="5" t="s">
         <v>272</v>
       </c>
-      <c r="D90" s="45">
+      <c r="D90" s="43">
         <v>18.63</v>
       </c>
       <c r="E90" s="22" t="s">
         <v>170</v>
       </c>
-      <c r="F90" s="46">
+      <c r="F90" s="44">
         <v>5</v>
       </c>
     </row>
@@ -3899,13 +3899,13 @@
       <c r="C91" s="5" t="s">
         <v>273</v>
       </c>
-      <c r="D91" s="45">
+      <c r="D91" s="43">
         <v>11.33</v>
       </c>
       <c r="E91" s="22" t="s">
         <v>171</v>
       </c>
-      <c r="F91" s="46">
+      <c r="F91" s="44">
         <v>6</v>
       </c>
     </row>
@@ -3919,14 +3919,14 @@
       <c r="C92" s="5" t="s">
         <v>264</v>
       </c>
-      <c r="D92" s="45">
+      <c r="D92" s="43">
         <v>22.97</v>
       </c>
       <c r="E92" s="22" t="s">
         <v>172</v>
       </c>
-      <c r="F92" s="46">
-        <v>15</v>
+      <c r="F92" s="44">
+        <v>12</v>
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.3">
@@ -3939,13 +3939,13 @@
       <c r="C93" s="5" t="s">
         <v>274</v>
       </c>
-      <c r="D93" s="45">
+      <c r="D93" s="43">
         <v>18.150000000000002</v>
       </c>
       <c r="E93" s="22" t="s">
         <v>173</v>
       </c>
-      <c r="F93" s="46">
+      <c r="F93" s="44">
         <v>5</v>
       </c>
     </row>
@@ -3959,13 +3959,13 @@
       <c r="C94" s="5" t="s">
         <v>275</v>
       </c>
-      <c r="D94" s="45">
+      <c r="D94" s="43">
         <v>12.83</v>
       </c>
       <c r="E94" s="22" t="s">
         <v>174</v>
       </c>
-      <c r="F94" s="46">
+      <c r="F94" s="44">
         <v>7</v>
       </c>
     </row>
@@ -3979,13 +3979,13 @@
       <c r="C95" s="5" t="s">
         <v>276</v>
       </c>
-      <c r="D95" s="45">
+      <c r="D95" s="43">
         <v>42.25</v>
       </c>
       <c r="E95" s="22" t="s">
         <v>175</v>
       </c>
-      <c r="F95" s="46">
+      <c r="F95" s="44">
         <v>11</v>
       </c>
     </row>
@@ -3999,14 +3999,14 @@
       <c r="C96" s="5" t="s">
         <v>277</v>
       </c>
-      <c r="D96" s="45">
-        <v>17.38</v>
+      <c r="D96" s="43">
+        <v>19.63</v>
       </c>
       <c r="E96" s="22" t="s">
         <v>176</v>
       </c>
-      <c r="F96" s="46">
-        <v>3</v>
+      <c r="F96" s="44">
+        <v>6</v>
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.3">
@@ -4019,14 +4019,14 @@
       <c r="C97" s="5" t="s">
         <v>278</v>
       </c>
-      <c r="D97" s="45">
-        <v>27.18</v>
+      <c r="D97" s="43">
+        <v>27.93</v>
       </c>
       <c r="E97" s="22" t="s">
         <v>177</v>
       </c>
-      <c r="F97" s="46">
-        <v>3</v>
+      <c r="F97" s="44">
+        <v>6</v>
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.3">
@@ -4039,13 +4039,13 @@
       <c r="C98" s="5" t="s">
         <v>279</v>
       </c>
-      <c r="D98" s="45">
+      <c r="D98" s="43">
         <v>34.51</v>
       </c>
       <c r="E98" s="22" t="s">
         <v>178</v>
       </c>
-      <c r="F98" s="46">
+      <c r="F98" s="44">
         <v>7</v>
       </c>
     </row>
@@ -4059,13 +4059,13 @@
       <c r="C99" s="5" t="s">
         <v>280</v>
       </c>
-      <c r="D99" s="45">
+      <c r="D99" s="43">
         <v>42.57</v>
       </c>
       <c r="E99" s="22" t="s">
         <v>179</v>
       </c>
-      <c r="F99" s="46">
+      <c r="F99" s="44">
         <v>7</v>
       </c>
     </row>
@@ -4079,13 +4079,13 @@
       <c r="C100" s="5" t="s">
         <v>281</v>
       </c>
-      <c r="D100" s="45">
+      <c r="D100" s="43">
         <v>21.68</v>
       </c>
       <c r="E100" s="22" t="s">
         <v>180</v>
       </c>
-      <c r="F100" s="46">
+      <c r="F100" s="44">
         <v>6</v>
       </c>
     </row>
@@ -4099,14 +4099,14 @@
       <c r="C101" s="5" t="s">
         <v>268</v>
       </c>
-      <c r="D101" s="45">
+      <c r="D101" s="43">
         <v>24.78</v>
       </c>
       <c r="E101" s="22" t="s">
         <v>181</v>
       </c>
-      <c r="F101" s="46">
-        <v>9</v>
+      <c r="F101" s="44">
+        <v>6</v>
       </c>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.3">
@@ -4119,13 +4119,13 @@
       <c r="C102" s="5" t="s">
         <v>266</v>
       </c>
-      <c r="D102" s="45">
+      <c r="D102" s="43">
         <v>16.63</v>
       </c>
       <c r="E102" s="22" t="s">
         <v>182</v>
       </c>
-      <c r="F102" s="46">
+      <c r="F102" s="44">
         <v>0</v>
       </c>
     </row>
@@ -4139,14 +4139,14 @@
       <c r="C103" s="5" t="s">
         <v>324</v>
       </c>
-      <c r="D103" s="45">
-        <v>19.72</v>
+      <c r="D103" s="43">
+        <v>16.04</v>
       </c>
       <c r="E103" s="22" t="s">
         <v>183</v>
       </c>
-      <c r="F103" s="46">
-        <v>12</v>
+      <c r="F103" s="44">
+        <v>3</v>
       </c>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.3">
@@ -4159,13 +4159,13 @@
       <c r="C104" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="D104" s="45">
+      <c r="D104" s="43">
         <v>33.01</v>
       </c>
       <c r="E104" s="22" t="s">
         <v>184</v>
       </c>
-      <c r="F104" s="46">
+      <c r="F104" s="44">
         <v>15</v>
       </c>
     </row>
@@ -4179,14 +4179,14 @@
       <c r="C105" s="5" t="s">
         <v>231</v>
       </c>
-      <c r="D105" s="35">
+      <c r="D105" s="45">
         <v>28.75</v>
       </c>
       <c r="E105" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="F105" s="36">
-        <v>7</v>
+      <c r="F105" s="46">
+        <v>2</v>
       </c>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.3">
@@ -4199,14 +4199,14 @@
       <c r="C106" s="5" t="s">
         <v>287</v>
       </c>
-      <c r="D106" s="35">
-        <v>58.82</v>
+      <c r="D106" s="45">
+        <v>64.59</v>
       </c>
       <c r="E106" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="F106" s="36">
-        <v>0</v>
+      <c r="F106" s="46">
+        <v>4</v>
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.3">
@@ -4219,14 +4219,14 @@
       <c r="C107" s="5" t="s">
         <v>288</v>
       </c>
-      <c r="D107" s="35">
-        <v>23.490000000000002</v>
+      <c r="D107" s="45">
+        <v>23.22</v>
       </c>
       <c r="E107" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="F107" s="36">
-        <v>1</v>
+      <c r="F107" s="46">
+        <v>6</v>
       </c>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.3">
@@ -4239,14 +4239,14 @@
       <c r="C108" s="5" t="s">
         <v>289</v>
       </c>
-      <c r="D108" s="35">
-        <v>59.9</v>
+      <c r="D108" s="45">
+        <v>59.5</v>
       </c>
       <c r="E108" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="F108" s="36">
-        <v>0</v>
+      <c r="F108" s="46">
+        <v>4</v>
       </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.3">
@@ -4286,7 +4286,7 @@
         <v>328</v>
       </c>
       <c r="F110" s="48">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.3">
@@ -4326,7 +4326,7 @@
         <v>330</v>
       </c>
       <c r="F112" s="48">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.3">
@@ -4346,7 +4346,7 @@
         <v>331</v>
       </c>
       <c r="F113" s="48">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.3">
@@ -4386,7 +4386,7 @@
         <v>333</v>
       </c>
       <c r="F115" s="48">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.3">
@@ -4484,7 +4484,7 @@
         <v>349</v>
       </c>
       <c r="F120" s="50">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.3">
@@ -4772,7 +4772,7 @@
         <v>364</v>
       </c>
       <c r="F135" s="50">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="136" spans="1:6" x14ac:dyDescent="0.3">
@@ -4792,7 +4792,7 @@
         <v>365</v>
       </c>
       <c r="F136" s="50">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="137" spans="1:6" x14ac:dyDescent="0.3">
@@ -4812,7 +4812,7 @@
         <v>366</v>
       </c>
       <c r="F137" s="50">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="138" spans="1:6" x14ac:dyDescent="0.3">
@@ -4888,7 +4888,7 @@
         <v>370</v>
       </c>
       <c r="F141" s="50">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="142" spans="1:6" x14ac:dyDescent="0.3">
@@ -4906,7 +4906,7 @@
         <v>371</v>
       </c>
       <c r="F142" s="50">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="143" spans="1:6" x14ac:dyDescent="0.3">
@@ -4926,7 +4926,7 @@
         <v>372</v>
       </c>
       <c r="F143" s="50">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="144" spans="1:6" x14ac:dyDescent="0.3">
@@ -4978,13 +4978,13 @@
         <v>468</v>
       </c>
       <c r="D146" s="49">
-        <v>8.14</v>
+        <v>8.6300000000000008</v>
       </c>
       <c r="E146" s="32" t="s">
         <v>375</v>
       </c>
       <c r="F146" s="50">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="147" spans="1:6" x14ac:dyDescent="0.3">
@@ -5042,7 +5042,7 @@
         <v>405</v>
       </c>
       <c r="F149" s="5">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="150" spans="1:6" x14ac:dyDescent="0.3">
@@ -5062,7 +5062,7 @@
         <v>438</v>
       </c>
       <c r="F150" s="52">
-        <v>280</v>
+        <v>205</v>
       </c>
     </row>
     <row r="151" spans="1:6" x14ac:dyDescent="0.3">
@@ -5170,7 +5170,7 @@
         <v>444</v>
       </c>
       <c r="F156" s="52">
-        <v>11</v>
+        <v>2</v>
       </c>
     </row>
     <row r="157" spans="1:6" x14ac:dyDescent="0.3">
@@ -5230,7 +5230,7 @@
         <v>447</v>
       </c>
       <c r="F159" s="52">
-        <v>130</v>
+        <v>105</v>
       </c>
     </row>
     <row r="160" spans="1:6" x14ac:dyDescent="0.3">
@@ -5250,7 +5250,7 @@
         <v>448</v>
       </c>
       <c r="F160" s="52">
-        <v>143</v>
+        <v>99</v>
       </c>
     </row>
     <row r="161" spans="1:6" x14ac:dyDescent="0.3">
@@ -5270,7 +5270,7 @@
         <v>449</v>
       </c>
       <c r="F161" s="52">
-        <v>248</v>
+        <v>198</v>
       </c>
     </row>
     <row r="162" spans="1:6" x14ac:dyDescent="0.3">
@@ -5290,7 +5290,7 @@
         <v>450</v>
       </c>
       <c r="F162" s="52">
-        <v>180</v>
+        <v>139</v>
       </c>
     </row>
     <row r="163" spans="1:6" x14ac:dyDescent="0.3">
@@ -5310,7 +5310,7 @@
         <v>451</v>
       </c>
       <c r="F163" s="52">
-        <v>0</v>
+        <v>-25</v>
       </c>
     </row>
     <row r="164" spans="1:6" x14ac:dyDescent="0.3">
@@ -5330,7 +5330,7 @@
         <v>452</v>
       </c>
       <c r="F164" s="52">
-        <v>35</v>
+        <v>24</v>
       </c>
     </row>
     <row r="165" spans="1:6" x14ac:dyDescent="0.3">

</xml_diff>